<commit_message>
sweep the two contrasts under every candidate label, plus F01
</commit_message>
<xml_diff>
--- a/03_Features/01_Responsiveness/c_data/01_label_audit.xlsx
+++ b/03_Features/01_Responsiveness/c_data/01_label_audit.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
     <t xml:space="preserve">trait</t>
   </si>
@@ -40,6 +40,18 @@
     <t xml:space="preserve">p</t>
   </si>
   <si>
+    <t xml:space="preserve">sd_change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mean_d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ci_lo_d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ci_hi_d</t>
+  </si>
+  <si>
     <t xml:space="preserve">comp_hypertrophy</t>
   </si>
   <si>
@@ -67,10 +79,7 @@
     <t xml:space="preserve">difference</t>
   </si>
   <si>
-    <t xml:space="preserve">sd_change</t>
-  </si>
-  <si>
-    <t xml:space="preserve">d</t>
+    <t xml:space="preserve">difference_d</t>
   </si>
   <si>
     <t xml:space="preserve">r</t>
@@ -481,10 +490,22 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B2" t="n">
         <v>16</v>
@@ -504,10 +525,22 @@
       <c r="G2" t="n">
         <v>0.0237957860659974</v>
       </c>
+      <c r="H2" t="n">
+        <v>8.61669271433845</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.628721503667539</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.0958591172775953</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1.16158389005748</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
         <v>16</v>
@@ -527,10 +560,22 @@
       <c r="G3" t="n">
         <v>0.67711459881652</v>
       </c>
+      <c r="H3" t="n">
+        <v>1423.6646446056</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-0.106164398036218</v>
+      </c>
+      <c r="J3" t="n">
+        <v>-0.639026784426162</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.426697988353726</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B4" t="n">
         <v>16</v>
@@ -550,10 +595,22 @@
       <c r="G4" t="n">
         <v>0.799239922163086</v>
       </c>
+      <c r="H4" t="n">
+        <v>1330.43532202496</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.0647222368306787</v>
+      </c>
+      <c r="J4" t="n">
+        <v>-0.468140149559265</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.597584623220623</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B5" t="n">
         <v>16</v>
@@ -573,10 +630,22 @@
       <c r="G5" t="n">
         <v>0.000423451596641191</v>
       </c>
+      <c r="H5" t="n">
+        <v>1.84624146014726</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1.12495442488565</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.592092038495707</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1.6578168112756</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B6" t="n">
         <v>16</v>
@@ -596,10 +665,22 @@
       <c r="G6" t="n">
         <v>0.0000724683159868194</v>
       </c>
+      <c r="H6" t="n">
+        <v>31.6611618022249</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1.35220874923773</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.819346362847788</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1.88507113562768</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B7" t="n">
         <v>15</v>
@@ -618,6 +699,18 @@
       </c>
       <c r="G7" t="n">
         <v>0.0000520917471123112</v>
+      </c>
+      <c r="H7" t="n">
+        <v>6.6246293696866</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1.47932804284017</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.925546501275304</v>
+      </c>
+      <c r="K7" t="n">
+        <v>2.03310958440504</v>
       </c>
     </row>
   </sheetData>
@@ -636,30 +729,42 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D1" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="G1" t="s">
-        <v>16</v>
-      </c>
-      <c r="H1" t="s">
-        <v>17</v>
+      <c r="I1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B2" t="n">
         <v>13.1</v>
@@ -671,21 +776,33 @@
         <v>15.365</v>
       </c>
       <c r="E2" t="n">
+        <v>11.6066667784424</v>
+      </c>
+      <c r="F2" t="n">
+        <v>19.1233332215576</v>
+      </c>
+      <c r="G2" t="n">
         <v>8.8348275720909</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
         <v>0.000000759141810025733</v>
       </c>
-      <c r="G2" t="n">
+      <c r="I2" t="n">
         <v>8.61669271433845</v>
       </c>
-      <c r="H2" t="n">
+      <c r="J2" t="n">
         <v>1.78316675659469</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1.34699787531341</v>
+      </c>
+      <c r="L2" t="n">
+        <v>2.21933563787597</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
         <v>889.5525</v>
@@ -697,21 +814,33 @@
         <v>2081.39</v>
       </c>
       <c r="E3" t="n">
+        <v>1024.04617601175</v>
+      </c>
+      <c r="F3" t="n">
+        <v>3138.73382398825</v>
+      </c>
+      <c r="G3" t="n">
         <v>4.30774757283746</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="n">
         <v>0.00111031808792229</v>
       </c>
-      <c r="G3" t="n">
+      <c r="I3" t="n">
         <v>1423.6646446056</v>
       </c>
-      <c r="H3" t="n">
+      <c r="J3" t="n">
         <v>1.4619945841084</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.719302948128941</v>
+      </c>
+      <c r="L3" t="n">
+        <v>2.20468622008785</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B4" t="n">
         <v>1043.16875</v>
@@ -723,21 +852,33 @@
         <v>1914.12</v>
       </c>
       <c r="E4" t="n">
+        <v>922.368440131609</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2905.87155986839</v>
+      </c>
+      <c r="G4" t="n">
         <v>4.15310320963433</v>
       </c>
-      <c r="F4" t="n">
+      <c r="H4" t="n">
         <v>0.00104585273562439</v>
       </c>
-      <c r="G4" t="n">
+      <c r="I4" t="n">
         <v>1330.43532202496</v>
       </c>
-      <c r="H4" t="n">
+      <c r="J4" t="n">
         <v>1.4387170637402</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.693283186985548</v>
+      </c>
+      <c r="L4" t="n">
+        <v>2.18415094049485</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B5" t="n">
         <v>3.012625</v>
@@ -749,21 +890,33 @@
         <v>1.871375</v>
       </c>
       <c r="E5" t="n">
+        <v>0.0606772738462712</v>
+      </c>
+      <c r="F5" t="n">
+        <v>3.68207272615373</v>
+      </c>
+      <c r="G5" t="n">
         <v>2.29850462171595</v>
       </c>
-      <c r="F5" t="n">
+      <c r="H5" t="n">
         <v>0.044028002060952</v>
       </c>
-      <c r="G5" t="n">
+      <c r="I5" t="n">
         <v>1.84624146014726</v>
       </c>
-      <c r="H5" t="n">
+      <c r="J5" t="n">
         <v>1.0136133546967</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.0328652969592783</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1.99436141243413</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B6" t="n">
         <v>45</v>
@@ -775,21 +928,33 @@
         <v>4.375</v>
       </c>
       <c r="E6" t="n">
+        <v>-30.6868921303313</v>
+      </c>
+      <c r="F6" t="n">
+        <v>39.4368921303313</v>
+      </c>
+      <c r="G6" t="n">
         <v>0.267675170823725</v>
       </c>
-      <c r="F6" t="n">
+      <c r="H6" t="n">
         <v>0.792860265103992</v>
       </c>
-      <c r="G6" t="n">
+      <c r="I6" t="n">
         <v>31.6611618022249</v>
       </c>
-      <c r="H6" t="n">
+      <c r="J6" t="n">
         <v>0.138181915980498</v>
+      </c>
+      <c r="K6" t="n">
+        <v>-0.969228240012812</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1.24559207197381</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B7" t="n">
         <v>10.7142857142857</v>
@@ -801,16 +966,28 @@
         <v>1.71428571428571</v>
       </c>
       <c r="E7" t="n">
+        <v>-5.84764848058783</v>
+      </c>
+      <c r="F7" t="n">
+        <v>9.27621990915926</v>
+      </c>
+      <c r="G7" t="n">
         <v>0.489829921346899</v>
       </c>
-      <c r="F7" t="n">
+      <c r="H7" t="n">
         <v>0.63242868562423</v>
       </c>
-      <c r="G7" t="n">
+      <c r="I7" t="n">
         <v>6.6246293696866</v>
       </c>
-      <c r="H7" t="n">
+      <c r="J7" t="n">
         <v>0.258774584753383</v>
+      </c>
+      <c r="K7" t="n">
+        <v>-0.882713304286255</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1.40026247379302</v>
       </c>
     </row>
   </sheetData>
@@ -829,15 +1006,15 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B2" t="n">
         <v>0.856004310667277</v>
@@ -848,7 +1025,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B3" t="n">
         <v>0.829021879743861</v>
@@ -859,7 +1036,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B4" t="n">
         <v>0.496807795570891</v>
@@ -870,7 +1047,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B5" t="n">
         <v>0.273744611777964</v>
@@ -881,7 +1058,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B6" t="n">
         <v>0.127677047329517</v>
@@ -906,16 +1083,16 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2">
@@ -948,28 +1125,28 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="H1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2">
@@ -977,7 +1154,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C2" t="n">
         <v>-118.837036895944</v>
@@ -1011,24 +1188,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B2" t="n">
         <v>32</v>
@@ -1045,7 +1222,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B3" t="n">
         <v>32</v>

</xml_diff>

<commit_message>
expand to ten phenotypes and add the acute contrast, still nothing there
</commit_message>
<xml_diff>
--- a/03_Features/01_Responsiveness/c_data/01_label_audit.xlsx
+++ b/03_Features/01_Responsiveness/c_data/01_label_audit.xlsx
@@ -11,13 +11,13 @@
     <sheet name="composite_structure" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="split_check" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="composite_modality" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="method_check" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="fibre_count_check" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t xml:space="preserve">trait</t>
   </si>
@@ -61,6 +61,15 @@
     <t xml:space="preserve">d_fcsa_II</t>
   </si>
   <si>
+    <t xml:space="preserve">d_fcsa_mixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_nfibre_mixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_nfibre_I</t>
+  </si>
+  <si>
     <t xml:space="preserve">d_mcsa</t>
   </si>
   <si>
@@ -82,6 +91,9 @@
     <t xml:space="preserve">difference_d</t>
   </si>
   <si>
+    <t xml:space="preserve">volume_load</t>
+  </si>
+  <si>
     <t xml:space="preserve">r</t>
   </si>
   <si>
@@ -130,10 +142,16 @@
     <t xml:space="preserve">quantity</t>
   </si>
   <si>
-    <t xml:space="preserve">mean_difference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sd_difference</t>
+    <t xml:space="preserve">area_median</t>
+  </si>
+  <si>
+    <t xml:space="preserve">count_median</t>
+  </si>
+  <si>
+    <t xml:space="preserve">r_area_count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">r_area_inverse_count</t>
   </si>
   <si>
     <t xml:space="preserve">fCSA_Mixed_Pre</t>
@@ -616,31 +634,31 @@
         <v>16</v>
       </c>
       <c r="C5" t="n">
-        <v>2.0769375</v>
+        <v>-23.9381250000001</v>
       </c>
       <c r="D5" t="n">
-        <v>1.09314486969388</v>
+        <v>-743.339148722331</v>
       </c>
       <c r="E5" t="n">
-        <v>3.06073013030612</v>
+        <v>695.462898722331</v>
       </c>
       <c r="F5" t="n">
-        <v>4.4998176995426</v>
+        <v>-0.0709241493552513</v>
       </c>
       <c r="G5" t="n">
-        <v>0.000423451596641191</v>
+        <v>0.944395096260056</v>
       </c>
       <c r="H5" t="n">
-        <v>1.84624146014726</v>
+        <v>1350.06906491591</v>
       </c>
       <c r="I5" t="n">
-        <v>1.12495442488565</v>
+        <v>-0.0177310373388128</v>
       </c>
       <c r="J5" t="n">
-        <v>0.592092038495707</v>
+        <v>-0.550593423728757</v>
       </c>
       <c r="K5" t="n">
-        <v>1.6578168112756</v>
+        <v>0.515131349051131</v>
       </c>
     </row>
     <row r="6">
@@ -651,31 +669,31 @@
         <v>16</v>
       </c>
       <c r="C6" t="n">
-        <v>42.8125</v>
+        <v>34.1875</v>
       </c>
       <c r="D6" t="n">
-        <v>25.9414577661883</v>
+        <v>-148.288547828447</v>
       </c>
       <c r="E6" t="n">
-        <v>59.6835422338117</v>
+        <v>216.663547828447</v>
       </c>
       <c r="F6" t="n">
-        <v>5.40883499695093</v>
+        <v>0.39933422608611</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0000724683159868194</v>
+        <v>0.695274924894311</v>
       </c>
       <c r="H6" t="n">
-        <v>31.6611618022249</v>
+        <v>342.444977332126</v>
       </c>
       <c r="I6" t="n">
-        <v>1.35220874923773</v>
+        <v>0.0998335565215276</v>
       </c>
       <c r="J6" t="n">
-        <v>0.819346362847788</v>
+        <v>-0.433028829868416</v>
       </c>
       <c r="K6" t="n">
-        <v>1.88507113562768</v>
+        <v>0.632695942911471</v>
       </c>
     </row>
     <row r="7">
@@ -683,33 +701,138 @@
         <v>16</v>
       </c>
       <c r="B7" t="n">
+        <v>16</v>
+      </c>
+      <c r="C7" t="n">
+        <v>15.8125</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-60.4513134737242</v>
+      </c>
+      <c r="E7" t="n">
+        <v>92.0763134737242</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.441933656396242</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.664842150377003</v>
+      </c>
+      <c r="H7" t="n">
+        <v>143.121029784818</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.110483414099061</v>
+      </c>
+      <c r="J7" t="n">
+        <v>-0.422378972290883</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.643345800489004</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" t="n">
+        <v>16</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2.0769375</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1.09314486969388</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3.06073013030612</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.4998176995426</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.000423451596641191</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1.84624146014726</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1.12495442488565</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.592092038495707</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1.6578168112756</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" t="n">
+        <v>16</v>
+      </c>
+      <c r="C9" t="n">
+        <v>42.8125</v>
+      </c>
+      <c r="D9" t="n">
+        <v>25.9414577661883</v>
+      </c>
+      <c r="E9" t="n">
+        <v>59.6835422338117</v>
+      </c>
+      <c r="F9" t="n">
+        <v>5.40883499695093</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.0000724683159868194</v>
+      </c>
+      <c r="H9" t="n">
+        <v>31.6611618022249</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1.35220874923773</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.819346362847788</v>
+      </c>
+      <c r="K9" t="n">
+        <v>1.88507113562768</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" t="n">
         <v>15</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C10" t="n">
         <v>9.8</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D10" t="n">
         <v>6.13140253535906</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E10" t="n">
         <v>13.4685974646409</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F10" t="n">
         <v>5.7294128734976</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G10" t="n">
         <v>0.0000520917471123112</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H10" t="n">
         <v>6.6246293696866</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I10" t="n">
         <v>1.47932804284017</v>
       </c>
-      <c r="J7" t="n">
+      <c r="J10" t="n">
         <v>0.925546501275304</v>
       </c>
-      <c r="K7" t="n">
+      <c r="K10" t="n">
         <v>2.03310958440504</v>
       </c>
     </row>
@@ -729,13 +852,13 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
@@ -753,7 +876,7 @@
         <v>7</v>
       </c>
       <c r="J1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="K1" t="s">
         <v>9</v>
@@ -881,37 +1004,37 @@
         <v>14</v>
       </c>
       <c r="B5" t="n">
-        <v>3.012625</v>
+        <v>914.04625</v>
       </c>
       <c r="C5" t="n">
-        <v>1.14125</v>
+        <v>-961.9225</v>
       </c>
       <c r="D5" t="n">
-        <v>1.871375</v>
+        <v>1875.96875</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0606772738462712</v>
+        <v>829.161161445729</v>
       </c>
       <c r="F5" t="n">
-        <v>3.68207272615373</v>
+        <v>2922.77633855427</v>
       </c>
       <c r="G5" t="n">
-        <v>2.29850462171595</v>
+        <v>3.8547341870158</v>
       </c>
       <c r="H5" t="n">
-        <v>0.044028002060952</v>
+        <v>0.00184410864144996</v>
       </c>
       <c r="I5" t="n">
-        <v>1.84624146014726</v>
+        <v>1350.06906491591</v>
       </c>
       <c r="J5" t="n">
-        <v>1.0136133546967</v>
+        <v>1.38953539396657</v>
       </c>
       <c r="K5" t="n">
-        <v>0.0328652969592783</v>
+        <v>0.614162032886351</v>
       </c>
       <c r="L5" t="n">
-        <v>1.99436141243413</v>
+        <v>2.16490875504678</v>
       </c>
     </row>
     <row r="6">
@@ -919,37 +1042,37 @@
         <v>15</v>
       </c>
       <c r="B6" t="n">
-        <v>45</v>
+        <v>-146.375</v>
       </c>
       <c r="C6" t="n">
-        <v>40.625</v>
+        <v>214.75</v>
       </c>
       <c r="D6" t="n">
-        <v>4.375</v>
+        <v>-361.125</v>
       </c>
       <c r="E6" t="n">
-        <v>-30.6868921303313</v>
+        <v>-681.005148034697</v>
       </c>
       <c r="F6" t="n">
-        <v>39.4368921303313</v>
+        <v>-41.2448519653032</v>
       </c>
       <c r="G6" t="n">
-        <v>0.267675170823725</v>
+        <v>-2.42940225348848</v>
       </c>
       <c r="H6" t="n">
-        <v>0.792860265103992</v>
+        <v>0.0297220587519294</v>
       </c>
       <c r="I6" t="n">
-        <v>31.6611618022249</v>
+        <v>342.444977332126</v>
       </c>
       <c r="J6" t="n">
-        <v>0.138181915980498</v>
+        <v>-1.05454897546871</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.969228240012812</v>
+        <v>-1.98865567642481</v>
       </c>
       <c r="L6" t="n">
-        <v>1.24559207197381</v>
+        <v>-0.120442274512618</v>
       </c>
     </row>
     <row r="7">
@@ -957,37 +1080,189 @@
         <v>16</v>
       </c>
       <c r="B7" t="n">
+        <v>-43.125</v>
+      </c>
+      <c r="C7" t="n">
+        <v>74.75</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-117.875</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-262.312740267144</v>
+      </c>
+      <c r="F7" t="n">
+        <v>26.5627402671441</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-1.75830614643652</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.101575049328966</v>
+      </c>
+      <c r="I7" t="n">
+        <v>143.121029784818</v>
+      </c>
+      <c r="J7" t="n">
+        <v>-0.823603632374816</v>
+      </c>
+      <c r="K7" t="n">
+        <v>-1.83280361147157</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.18559634672194</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" t="n">
+        <v>3.012625</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1.14125</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1.871375</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.0606772738462712</v>
+      </c>
+      <c r="F8" t="n">
+        <v>3.68207272615373</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2.29850462171595</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.044028002060952</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1.84624146014726</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1.0136133546967</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.0328652969592783</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1.99436141243413</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" t="n">
+        <v>45</v>
+      </c>
+      <c r="C9" t="n">
+        <v>40.625</v>
+      </c>
+      <c r="D9" t="n">
+        <v>4.375</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-30.6868921303313</v>
+      </c>
+      <c r="F9" t="n">
+        <v>39.4368921303313</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.267675170823725</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.792860265103992</v>
+      </c>
+      <c r="I9" t="n">
+        <v>31.6611618022249</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.138181915980498</v>
+      </c>
+      <c r="K9" t="n">
+        <v>-0.969228240012812</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1.24559207197381</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" t="n">
         <v>10.7142857142857</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C10" t="n">
         <v>9</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D10" t="n">
         <v>1.71428571428571</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E10" t="n">
         <v>-5.84764848058783</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F10" t="n">
         <v>9.27621990915926</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G10" t="n">
         <v>0.489829921346899</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H10" t="n">
         <v>0.63242868562423</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I10" t="n">
         <v>6.6246293696866</v>
       </c>
-      <c r="J7" t="n">
+      <c r="J10" t="n">
         <v>0.258774584753383</v>
       </c>
-      <c r="K7" t="n">
+      <c r="K10" t="n">
         <v>-0.882713304286255</v>
       </c>
-      <c r="L7" t="n">
+      <c r="L10" t="n">
         <v>1.40026247379302</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" t="n">
+        <v>126078.625</v>
+      </c>
+      <c r="C11" t="n">
+        <v>139466.25</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-13387.625</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-74034.0779795756</v>
+      </c>
+      <c r="F11" t="n">
+        <v>47258.8279795756</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-0.474638896928969</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.642554614226018</v>
+      </c>
+      <c r="I11" t="n">
+        <v>54935.7455080858</v>
+      </c>
+      <c r="J11" t="n">
+        <v>-0.243696064851428</v>
+      </c>
+      <c r="K11" t="n">
+        <v>-1.34764855368494</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.860256423982082</v>
       </c>
     </row>
   </sheetData>
@@ -1006,10 +1281,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2">
@@ -1039,10 +1314,10 @@
         <v>14</v>
       </c>
       <c r="B4" t="n">
-        <v>0.496807795570891</v>
+        <v>0.835177563982897</v>
       </c>
       <c r="C4" t="n">
-        <v>0.246817985740008</v>
+        <v>0.697521563380406</v>
       </c>
     </row>
     <row r="5">
@@ -1050,10 +1325,10 @@
         <v>15</v>
       </c>
       <c r="B5" t="n">
-        <v>0.273744611777964</v>
+        <v>-0.600282058411429</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0749361124774681</v>
+        <v>0.360338549650662</v>
       </c>
     </row>
     <row r="6">
@@ -1061,10 +1336,54 @@
         <v>16</v>
       </c>
       <c r="B6" t="n">
+        <v>-0.489823092226803</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.239926661678627</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.496807795570891</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.246817985740008</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.273744611777964</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.0749361124774681</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="n">
         <v>0.127677047329517</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C9" t="n">
         <v>0.0163014284147838</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.0433581560331737</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.00187992969459705</v>
       </c>
     </row>
   </sheetData>
@@ -1083,16 +1402,16 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D1" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2">
@@ -1125,28 +1444,28 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B1" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C1" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="E1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F1" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H1" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2">
@@ -1154,7 +1473,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C2" t="n">
         <v>-118.837036895944</v>
@@ -1188,53 +1507,62 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="D1" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="E1" t="s">
-        <v>38</v>
+        <v>43</v>
+      </c>
+      <c r="F1" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="B2" t="n">
         <v>32</v>
       </c>
       <c r="C2" t="n">
+        <v>6179.225</v>
+      </c>
+      <c r="D2" t="n">
+        <v>517</v>
+      </c>
+      <c r="E2" t="n">
         <v>-0.629724099658717</v>
       </c>
-      <c r="D2" t="n">
-        <v>-5660.3153125</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1635.38190163049</v>
+      <c r="F2" t="n">
+        <v>0.542264187708715</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B3" t="n">
         <v>32</v>
       </c>
       <c r="C3" t="n">
+        <v>5688.12</v>
+      </c>
+      <c r="D3" t="n">
+        <v>184</v>
+      </c>
+      <c r="E3" t="n">
         <v>-0.437134859266442</v>
       </c>
-      <c r="D3" t="n">
-        <v>-5689.923125</v>
-      </c>
-      <c r="E3" t="n">
-        <v>1380.39937763803</v>
+      <c r="F3" t="n">
+        <v>0.254587181570893</v>
       </c>
     </row>
   </sheetData>

</xml_diff>